<commit_message>
Update 711285 - MSCI AC Asia ex Japan ex China Index .xlsx
</commit_message>
<xml_diff>
--- a/data/711285 - MSCI AC Asia ex Japan ex China Index .xlsx
+++ b/data/711285 - MSCI AC Asia ex Japan ex China Index .xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3977" uniqueCount="3976">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4001" uniqueCount="4000">
   <si>
     <t>Index Level:</t>
   </si>
@@ -11939,6 +11939,78 @@
   </si>
   <si>
     <t>2026-03-27</t>
+  </si>
+  <si>
+    <t>2026-03-30</t>
+  </si>
+  <si>
+    <t>2026-03-31</t>
+  </si>
+  <si>
+    <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>2026-04-02</t>
+  </si>
+  <si>
+    <t>2026-04-03</t>
+  </si>
+  <si>
+    <t>2026-04-06</t>
+  </si>
+  <si>
+    <t>2026-04-07</t>
+  </si>
+  <si>
+    <t>2026-04-08</t>
+  </si>
+  <si>
+    <t>2026-04-09</t>
+  </si>
+  <si>
+    <t>2026-04-10</t>
+  </si>
+  <si>
+    <t>2026-04-13</t>
+  </si>
+  <si>
+    <t>2026-04-14</t>
+  </si>
+  <si>
+    <t>2026-04-15</t>
+  </si>
+  <si>
+    <t>2026-04-16</t>
+  </si>
+  <si>
+    <t>2026-04-17</t>
+  </si>
+  <si>
+    <t>2026-04-20</t>
+  </si>
+  <si>
+    <t>2026-04-21</t>
+  </si>
+  <si>
+    <t>2026-04-22</t>
+  </si>
+  <si>
+    <t>2026-04-23</t>
+  </si>
+  <si>
+    <t>2026-04-24</t>
+  </si>
+  <si>
+    <t>2026-04-27</t>
+  </si>
+  <si>
+    <t>2026-04-28</t>
+  </si>
+  <si>
+    <t>2026-04-29</t>
+  </si>
+  <si>
+    <t>2026-04-30</t>
   </si>
 </sst>
 </file>
@@ -12324,7 +12396,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A3:E3961"/>
+  <dimension ref="A3:E3985"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -44049,6 +44121,198 @@
         <v>7363.294877</v>
       </c>
     </row>
+    <row r="3962" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3962" t="s">
+        <v>3976</v>
+      </c>
+      <c r="B3962">
+        <v>7184.029593</v>
+      </c>
+    </row>
+    <row r="3963" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3963" t="s">
+        <v>3977</v>
+      </c>
+      <c r="B3963">
+        <v>7028.177913</v>
+      </c>
+    </row>
+    <row r="3964" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3964" t="s">
+        <v>3978</v>
+      </c>
+      <c r="B3964">
+        <v>7422.150293</v>
+      </c>
+    </row>
+    <row r="3965" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3965" t="s">
+        <v>3979</v>
+      </c>
+      <c r="B3965">
+        <v>7262.684496</v>
+      </c>
+    </row>
+    <row r="3966" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3966" t="s">
+        <v>3980</v>
+      </c>
+      <c r="B3966">
+        <v>7321.060401</v>
+      </c>
+    </row>
+    <row r="3967" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3967" t="s">
+        <v>3981</v>
+      </c>
+      <c r="B3967">
+        <v>7391.048724</v>
+      </c>
+    </row>
+    <row r="3968" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3968" t="s">
+        <v>3982</v>
+      </c>
+      <c r="B3968">
+        <v>7487.5789</v>
+      </c>
+    </row>
+    <row r="3969" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3969" t="s">
+        <v>3983</v>
+      </c>
+      <c r="B3969">
+        <v>7947.057774</v>
+      </c>
+    </row>
+    <row r="3970" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3970" t="s">
+        <v>3984</v>
+      </c>
+      <c r="B3970">
+        <v>7881.854107</v>
+      </c>
+    </row>
+    <row r="3971" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3971" t="s">
+        <v>3985</v>
+      </c>
+      <c r="B3971">
+        <v>7995.80581</v>
+      </c>
+    </row>
+    <row r="3972" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3972" t="s">
+        <v>3986</v>
+      </c>
+      <c r="B3972">
+        <v>7917.370498</v>
+      </c>
+    </row>
+    <row r="3973" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3973" t="s">
+        <v>3987</v>
+      </c>
+      <c r="B3973">
+        <v>8098.094143</v>
+      </c>
+    </row>
+    <row r="3974" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3974" t="s">
+        <v>3988</v>
+      </c>
+      <c r="B3974">
+        <v>8232.206276</v>
+      </c>
+    </row>
+    <row r="3975" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3975" t="s">
+        <v>3989</v>
+      </c>
+      <c r="B3975">
+        <v>8331.571494</v>
+      </c>
+    </row>
+    <row r="3976" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3976" t="s">
+        <v>3990</v>
+      </c>
+      <c r="B3976">
+        <v>8264.448265</v>
+      </c>
+    </row>
+    <row r="3977" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3977" t="s">
+        <v>3991</v>
+      </c>
+      <c r="B3977">
+        <v>8305.659868</v>
+      </c>
+    </row>
+    <row r="3978" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3978" t="s">
+        <v>3992</v>
+      </c>
+      <c r="B3978">
+        <v>8453.280994</v>
+      </c>
+    </row>
+    <row r="3979" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3979" t="s">
+        <v>3993</v>
+      </c>
+      <c r="B3979">
+        <v>8446.773237</v>
+      </c>
+    </row>
+    <row r="3980" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3980" t="s">
+        <v>3994</v>
+      </c>
+      <c r="B3980">
+        <v>8435.718475</v>
+      </c>
+    </row>
+    <row r="3981" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3981" t="s">
+        <v>3995</v>
+      </c>
+      <c r="B3981">
+        <v>8527.656021</v>
+      </c>
+    </row>
+    <row r="3982" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3982" t="s">
+        <v>3996</v>
+      </c>
+      <c r="B3982">
+        <v>8710.70168</v>
+      </c>
+    </row>
+    <row r="3983" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3983" t="s">
+        <v>3997</v>
+      </c>
+      <c r="B3983">
+        <v>8668.169177</v>
+      </c>
+    </row>
+    <row r="3984" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3984" t="s">
+        <v>3998</v>
+      </c>
+      <c r="B3984">
+        <v>8651.679157</v>
+      </c>
+    </row>
+    <row r="3985" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3985" t="s">
+        <v>3999</v>
+      </c>
+      <c r="B3985">
+        <v>8541.209009</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>